<commit_message>
Update workbook to corrected v4 numbers
Regenerated all engine statistics from the honest baseline: matrix v4
(conditional-duration S, D-cell gold, R momentum tilt), monthly-only
execution, no retracted intra-month mechanisms. Evidence table now
CONS 9.5%/1.32/-11, MOD 14.4%/1.43/-16, AGG 22.7%/1.12/-36, VAGG
31.0%/1.10/-50. Data-sheet and Statistics labels updated to describe
the v4 monthly-only basis. Verified vs Python replication (glide 25->65
at 25% haircut + 24% ST tax: ~$12.4M on $2.59M contributed).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1598,7 +1598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Jun 2007 – Aug 2026 daily data, dividends included. Leveraged instruments simulated pre-2010. Forward validation: paper/ledger.csv (monthly, automated).</t>
+          <t>Matrix v4 (conditional-duration S, D-cell gold, R momentum tilt), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
         </is>
       </c>
     </row>
@@ -1683,34 +1683,34 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>0.0837</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>1.1858</v>
+        <v>1.3173</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>0.8632</v>
+        <v>0.9536</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>-0.1306</v>
+        <v>-0.1059</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>0.1749</v>
+        <v>0.1604</v>
       </c>
       <c r="G6" s="18" t="n">
-        <v>0.1381</v>
+        <v>0.1315</v>
       </c>
       <c r="H6" s="18" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.1228</v>
       </c>
       <c r="I6" s="18" t="n">
-        <v>-0.0127</v>
+        <v>0.021</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.1949</v>
+        <v>0.204</v>
       </c>
       <c r="K6" s="18" t="n">
-        <v>0.1357</v>
+        <v>0.1268</v>
       </c>
     </row>
     <row r="7">
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>0.1327</v>
+        <v>0.1443</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>1.3476</v>
+        <v>1.4307</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>0.9798</v>
+        <v>1.0503</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>-0.1496</v>
+        <v>-0.16</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.3065</v>
+        <v>0.3077</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>0.1541</v>
+        <v>0.1133</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>0.2216</v>
+        <v>0.2458</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>-0.0292</v>
+        <v>0.0221</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>0.2553</v>
+        <v>0.2703</v>
       </c>
       <c r="K7" s="20" t="n">
-        <v>0.1916</v>
+        <v>0.1771</v>
       </c>
     </row>
     <row r="8">
@@ -1757,34 +1757,34 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>0.1985</v>
+        <v>0.2271</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>1.0121</v>
+        <v>1.122</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>0.7635</v>
+        <v>0.878</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0.365</v>
+        <v>-0.3565</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>0.5868</v>
+        <v>0.6299</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>0.33</v>
+        <v>0.2365</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.6318</v>
+        <v>0.6504</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0.2428</v>
+        <v>-0.2259</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.3696</v>
+        <v>0.4798</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>0.2083</v>
+        <v>0.2039</v>
       </c>
     </row>
     <row r="9">
@@ -1794,34 +1794,34 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>0.267</v>
+        <v>0.3096</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.0056</v>
+        <v>1.1049</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>0.7679</v>
+        <v>0.8754</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>-0.5102</v>
+        <v>-0.5002</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.8663</v>
+        <v>0.96</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>0.5061</v>
+        <v>0.3016</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>0.9036999999999999</v>
+        <v>0.9754</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>-0.3465</v>
+        <v>-0.3142</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>0.4406</v>
+        <v>0.5814</v>
       </c>
       <c r="K9" s="20" t="n">
-        <v>0.3146</v>
+        <v>0.3244</v>
       </c>
     </row>
     <row r="10">
@@ -18022,7 +18022,7 @@
     <row r="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Model Data — per-regime return statistics (v2 rotation backtest, Jun 2007–Aug 2026)</t>
+          <t>Model Data — per-regime return statistics (matrix v4, monthly-only execution, Jun 2007–Aug 2026)</t>
         </is>
       </c>
     </row>
@@ -18073,16 +18073,16 @@
         </is>
       </c>
       <c r="B6" s="55" t="n">
-        <v>0.00731</v>
+        <v>0.00726</v>
       </c>
       <c r="C6" s="55" t="n">
-        <v>0.00769</v>
+        <v>0.00796</v>
       </c>
       <c r="D6" s="55" t="n">
-        <v>-0.00047</v>
+        <v>0.00399</v>
       </c>
       <c r="E6" s="55" t="n">
-        <v>0.007820000000000001</v>
+        <v>0.01116</v>
       </c>
     </row>
     <row r="7">
@@ -18092,16 +18092,16 @@
         </is>
       </c>
       <c r="B7" s="55" t="n">
-        <v>0.01397</v>
+        <v>0.01392</v>
       </c>
       <c r="C7" s="55" t="n">
-        <v>0.01033</v>
+        <v>0.01076</v>
       </c>
       <c r="D7" s="55" t="n">
-        <v>-0.0011</v>
+        <v>0.00463</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>0.01283</v>
+        <v>0.01446</v>
       </c>
     </row>
     <row r="8">
@@ -18114,13 +18114,13 @@
         <v>0.03406</v>
       </c>
       <c r="C8" s="55" t="n">
-        <v>0.01138</v>
+        <v>0.01205</v>
       </c>
       <c r="D8" s="55" t="n">
-        <v>-0.00554</v>
+        <v>0.00528</v>
       </c>
       <c r="E8" s="55" t="n">
-        <v>0.01183</v>
+        <v>0.0167</v>
       </c>
     </row>
     <row r="9">
@@ -18133,13 +18133,13 @@
         <v>0.05004</v>
       </c>
       <c r="C9" s="55" t="n">
-        <v>0.01556</v>
+        <v>0.01622</v>
       </c>
       <c r="D9" s="55" t="n">
-        <v>-0.00698</v>
+        <v>0.00593</v>
       </c>
       <c r="E9" s="55" t="n">
-        <v>0.01445</v>
+        <v>0.02286</v>
       </c>
     </row>
     <row r="11">
@@ -18182,16 +18182,16 @@
         </is>
       </c>
       <c r="B13" s="55" t="n">
-        <v>0.01765</v>
+        <v>0.01763</v>
       </c>
       <c r="C13" s="55" t="n">
-        <v>0.0223</v>
+        <v>0.02288</v>
       </c>
       <c r="D13" s="55" t="n">
-        <v>0.01283</v>
+        <v>0.01537</v>
       </c>
       <c r="E13" s="55" t="n">
-        <v>0.0278</v>
+        <v>0.03214</v>
       </c>
     </row>
     <row r="14">
@@ -18201,16 +18201,16 @@
         </is>
       </c>
       <c r="B14" s="55" t="n">
-        <v>0.03064</v>
+        <v>0.0307</v>
       </c>
       <c r="C14" s="55" t="n">
-        <v>0.03189</v>
+        <v>0.03269</v>
       </c>
       <c r="D14" s="55" t="n">
-        <v>0.01504</v>
+        <v>0.01819</v>
       </c>
       <c r="E14" s="55" t="n">
-        <v>0.03919</v>
+        <v>0.03913</v>
       </c>
     </row>
     <row r="15">
@@ -18223,13 +18223,13 @@
         <v>0.09061</v>
       </c>
       <c r="C15" s="55" t="n">
-        <v>0.04874</v>
+        <v>0.04889</v>
       </c>
       <c r="D15" s="55" t="n">
-        <v>0.02913</v>
+        <v>0.02114</v>
       </c>
       <c r="E15" s="55" t="n">
-        <v>0.0717</v>
+        <v>0.05551</v>
       </c>
     </row>
     <row r="16">
@@ -18242,13 +18242,13 @@
         <v>0.13741</v>
       </c>
       <c r="C16" s="55" t="n">
-        <v>0.06776</v>
+        <v>0.06826</v>
       </c>
       <c r="D16" s="55" t="n">
-        <v>0.03462</v>
+        <v>0.02416</v>
       </c>
       <c r="E16" s="55" t="n">
-        <v>0.1052</v>
+        <v>0.07714</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Refresh GrowthProjection.xlsx to matrix v6; GDX swap rejected, gold stays
- evidence.json tier rows + projection_stats.json regenerated from the
  v6 engine (shorts ON); convention check reproduces the stored SPY
  benchmark row to 4 decimals, keeping tiers and benchmarks on one
  identical method
- workbook Data sheet: per-regime monthly stats now include the short
  sleeves (MOD S 0.46->0.65%/mo, D 1.45->1.78%/mo); Statistics rows
  updated; version strings v4->v6
- GDX-for-GLD candidate rejected by user decision: bullion stays in
  every D-cell (incomplete pre-2007 two-sample leg was the weakness)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1144,7 +1144,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Age-based risk glide with regime-conditional return engine  |  Backtest Jun 2007–Aug 2026  |  Prepared August 20, 2026  |  Forward ledger live</t>
+          <t>Age-based risk glide with regime-conditional return engine  |  Backtest Jun 2007–Aug 2026  |  Prepared August 21, 2026  |  Forward ledger live</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Matrix v4 (conditional-duration S, D-cell gold, R momentum tilt), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
+          <t>Matrix v6 (conditional-duration S, D-cell gold, R momentum tilt, regime-gated short book: oil in Deflation + energy equities in Stagflation behind a global include-shorts switch), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
         </is>
       </c>
     </row>
@@ -1683,34 +1683,34 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.09669999999999999</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>1.3173</v>
+        <v>1.5983</v>
       </c>
       <c r="D6" s="19" t="n">
-        <v>0.9536</v>
+        <v>1.1522</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>-0.1059</v>
+        <v>-0.1021</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>0.1604</v>
+        <v>0.1671</v>
       </c>
       <c r="G6" s="18" t="n">
-        <v>0.1315</v>
+        <v>0.1382</v>
       </c>
       <c r="H6" s="18" t="n">
-        <v>0.1228</v>
+        <v>0.1297</v>
       </c>
       <c r="I6" s="18" t="n">
-        <v>0.021</v>
+        <v>0.0187</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.204</v>
+        <v>0.2063</v>
       </c>
       <c r="K6" s="18" t="n">
-        <v>0.1268</v>
+        <v>0.1283</v>
       </c>
     </row>
     <row r="7">
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>0.1443</v>
+        <v>0.1528</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>1.4307</v>
+        <v>1.7335</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>1.0503</v>
+        <v>1.2456</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>-0.16</v>
+        <v>-0.1431</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.3077</v>
+        <v>0.2789</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>0.1133</v>
+        <v>0.2075</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>0.2458</v>
+        <v>0.36</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>0.0221</v>
+        <v>0.0002</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>0.2703</v>
+        <v>0.2861</v>
       </c>
       <c r="K7" s="20" t="n">
-        <v>0.1771</v>
+        <v>0.1833</v>
       </c>
     </row>
     <row r="8">
@@ -1757,34 +1757,34 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>0.2271</v>
+        <v>0.2408</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>1.122</v>
+        <v>1.2244</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>0.878</v>
+        <v>0.9427</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0.3565</v>
+        <v>-0.3375</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>0.6299</v>
+        <v>0.5864</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>0.2365</v>
+        <v>0.38</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.6504</v>
+        <v>0.9095</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0.2259</v>
+        <v>-0.2531</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.4798</v>
+        <v>0.4978</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>0.2039</v>
+        <v>0.217</v>
       </c>
     </row>
     <row r="9">
@@ -1794,34 +1794,34 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>0.3096</v>
+        <v>0.338</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.1049</v>
+        <v>1.1173</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>0.8754</v>
+        <v>0.8657</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>-0.5002</v>
+        <v>-0.489</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.96</v>
+        <v>0.9979</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>0.3016</v>
+        <v>0.4634</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>0.9754</v>
+        <v>1.1018</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>-0.3142</v>
+        <v>-0.3122</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>0.5814</v>
+        <v>0.6196</v>
       </c>
       <c r="K9" s="20" t="n">
-        <v>0.3244</v>
+        <v>0.4992</v>
       </c>
     </row>
     <row r="10">
@@ -1834,16 +1834,16 @@
         <v>0.1082</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>0.6697</v>
+        <v>0.6728</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>0.5458</v>
+        <v>0.5484</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>-0.5518999999999999</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>1.0002</v>
+        <v>1</v>
       </c>
       <c r="G10" s="18" t="n">
         <v>-0.368</v>
@@ -1871,16 +1871,16 @@
         <v>0.1625</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>0.9358</v>
+        <v>0.9438</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.7202</v>
+        <v>0.7264</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>-0.534</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>1.0467</v>
+        <v>1.0465</v>
       </c>
       <c r="G11" s="18" t="n">
         <v>-0.4173</v>
@@ -18022,7 +18022,7 @@
     <row r="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Model Data — per-regime return statistics (matrix v4, monthly-only execution, Jun 2007–Aug 2026)</t>
+          <t>Model Data — per-regime return statistics (matrix v6, monthly-only execution, Jun 2007–Aug 2026)</t>
         </is>
       </c>
     </row>
@@ -18073,16 +18073,16 @@
         </is>
       </c>
       <c r="B6" s="55" t="n">
-        <v>0.00726</v>
+        <v>0.00731</v>
       </c>
       <c r="C6" s="55" t="n">
-        <v>0.00796</v>
+        <v>0.00805</v>
       </c>
       <c r="D6" s="55" t="n">
-        <v>0.00399</v>
+        <v>0.00398</v>
       </c>
       <c r="E6" s="55" t="n">
-        <v>0.01116</v>
+        <v>0.01164</v>
       </c>
     </row>
     <row r="7">
@@ -18092,16 +18092,16 @@
         </is>
       </c>
       <c r="B7" s="55" t="n">
-        <v>0.01392</v>
+        <v>0.01397</v>
       </c>
       <c r="C7" s="55" t="n">
-        <v>0.01076</v>
+        <v>0.01084</v>
       </c>
       <c r="D7" s="55" t="n">
-        <v>0.00463</v>
+        <v>0.00648</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>0.01446</v>
+        <v>0.01783</v>
       </c>
     </row>
     <row r="8">
@@ -18114,13 +18114,13 @@
         <v>0.03406</v>
       </c>
       <c r="C8" s="55" t="n">
-        <v>0.01205</v>
+        <v>0.01229</v>
       </c>
       <c r="D8" s="55" t="n">
-        <v>0.00528</v>
+        <v>0.00804</v>
       </c>
       <c r="E8" s="55" t="n">
-        <v>0.0167</v>
+        <v>0.02193</v>
       </c>
     </row>
     <row r="9">
@@ -18133,13 +18133,13 @@
         <v>0.05004</v>
       </c>
       <c r="C9" s="55" t="n">
-        <v>0.01622</v>
+        <v>0.01867</v>
       </c>
       <c r="D9" s="55" t="n">
-        <v>0.00593</v>
+        <v>0.00869</v>
       </c>
       <c r="E9" s="55" t="n">
-        <v>0.02286</v>
+        <v>0.02982</v>
       </c>
     </row>
     <row r="11">
@@ -18182,16 +18182,16 @@
         </is>
       </c>
       <c r="B13" s="55" t="n">
-        <v>0.01763</v>
+        <v>0.01765</v>
       </c>
       <c r="C13" s="55" t="n">
-        <v>0.02288</v>
+        <v>0.02286</v>
       </c>
       <c r="D13" s="55" t="n">
-        <v>0.01537</v>
+        <v>0.01519</v>
       </c>
       <c r="E13" s="55" t="n">
-        <v>0.03214</v>
+        <v>0.0323</v>
       </c>
     </row>
     <row r="14">
@@ -18201,16 +18201,16 @@
         </is>
       </c>
       <c r="B14" s="55" t="n">
-        <v>0.0307</v>
+        <v>0.03064</v>
       </c>
       <c r="C14" s="55" t="n">
-        <v>0.03269</v>
+        <v>0.0327</v>
       </c>
       <c r="D14" s="55" t="n">
-        <v>0.01819</v>
+        <v>0.02411</v>
       </c>
       <c r="E14" s="55" t="n">
-        <v>0.03913</v>
+        <v>0.04132</v>
       </c>
     </row>
     <row r="15">
@@ -18223,13 +18223,13 @@
         <v>0.09061</v>
       </c>
       <c r="C15" s="55" t="n">
-        <v>0.04889</v>
+        <v>0.04896</v>
       </c>
       <c r="D15" s="55" t="n">
-        <v>0.02114</v>
+        <v>0.03079</v>
       </c>
       <c r="E15" s="55" t="n">
-        <v>0.05551</v>
+        <v>0.06388000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -18242,13 +18242,13 @@
         <v>0.13741</v>
       </c>
       <c r="C16" s="55" t="n">
-        <v>0.06826</v>
+        <v>0.07905</v>
       </c>
       <c r="D16" s="55" t="n">
-        <v>0.02416</v>
+        <v>0.03353</v>
       </c>
       <c r="E16" s="55" t="n">
-        <v>0.07714</v>
+        <v>0.08375</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Deployment runbook + workbook defaults for updated capital/contributions
- DEPLOYMENT.md: preconditions, day-1 procedure, monthly routine,
  live short-book handling, scope, and honest self-measurement
- GrowthProjection.xlsx: starting balance 11k, year-1 contribution 900,
  schedule ramp now starts from the year-1 base (+12%/yr to yr 15,
  +8%/yr after)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1184,7 +1184,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>8000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="8">
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="9">
@@ -17596,7 +17596,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>650</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="21">
@@ -17606,7 +17606,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>800</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="22">
@@ -17616,7 +17616,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>900</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="23">
@@ -17626,7 +17626,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>1000</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="24">
@@ -17636,7 +17636,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>1125</v>
+        <v>1575</v>
       </c>
     </row>
     <row r="25">
@@ -17646,7 +17646,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>1250</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="26">
@@ -17656,7 +17656,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="27">
@@ -17666,7 +17666,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>1575</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="28">
@@ -17676,7 +17676,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>1775</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="29">
@@ -17686,7 +17686,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>1975</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="30">
@@ -17696,7 +17696,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>2225</v>
+        <v>3125</v>
       </c>
     </row>
     <row r="31">
@@ -17706,7 +17706,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>2475</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="32">
@@ -17716,7 +17716,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>2775</v>
+        <v>3925</v>
       </c>
     </row>
     <row r="33">
@@ -17726,7 +17726,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>3125</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="34">
@@ -17736,7 +17736,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>3375</v>
+        <v>4750</v>
       </c>
     </row>
     <row r="35">
@@ -17746,7 +17746,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>3625</v>
+        <v>5125</v>
       </c>
     </row>
     <row r="36">
@@ -17756,7 +17756,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>3925</v>
+        <v>5550</v>
       </c>
     </row>
     <row r="37">
@@ -17766,7 +17766,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>4250</v>
+        <v>5975</v>
       </c>
     </row>
     <row r="38">
@@ -17776,7 +17776,7 @@
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>4575</v>
+        <v>6475</v>
       </c>
     </row>
     <row r="39">
@@ -17786,7 +17786,7 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>4950</v>
+        <v>6975</v>
       </c>
     </row>
     <row r="40">
@@ -17796,7 +17796,7 @@
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>5350</v>
+        <v>7550</v>
       </c>
     </row>
     <row r="41">
@@ -17806,7 +17806,7 @@
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>5775</v>
+        <v>8150</v>
       </c>
     </row>
     <row r="42">
@@ -17816,7 +17816,7 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>6225</v>
+        <v>8800</v>
       </c>
     </row>
     <row r="43">
@@ -17826,7 +17826,7 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>6725</v>
+        <v>9500</v>
       </c>
     </row>
     <row r="44">
@@ -17836,7 +17836,7 @@
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>7275</v>
+        <v>10250</v>
       </c>
     </row>
     <row r="45">
@@ -17846,7 +17846,7 @@
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>7850</v>
+        <v>11075</v>
       </c>
     </row>
     <row r="46">
@@ -17856,7 +17856,7 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>8475</v>
+        <v>11950</v>
       </c>
     </row>
     <row r="47">
@@ -17866,7 +17866,7 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>9150</v>
+        <v>12925</v>
       </c>
     </row>
     <row r="48">
@@ -17876,7 +17876,7 @@
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>9875</v>
+        <v>13950</v>
       </c>
     </row>
     <row r="49">
@@ -17886,7 +17886,7 @@
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>10675</v>
+        <v>15075</v>
       </c>
     </row>
     <row r="50">
@@ -17896,7 +17896,7 @@
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>11525</v>
+        <v>16275</v>
       </c>
     </row>
     <row r="51">
@@ -17906,7 +17906,7 @@
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>12450</v>
+        <v>17575</v>
       </c>
     </row>
     <row r="52">
@@ -17916,7 +17916,7 @@
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>13450</v>
+        <v>18975</v>
       </c>
     </row>
     <row r="53">
@@ -17926,7 +17926,7 @@
         </is>
       </c>
       <c r="B53" s="7" t="n">
-        <v>14525</v>
+        <v>20500</v>
       </c>
     </row>
     <row r="54">
@@ -17936,7 +17936,7 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>15700</v>
+        <v>22150</v>
       </c>
     </row>
     <row r="55">
@@ -17946,7 +17946,7 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>16950</v>
+        <v>23900</v>
       </c>
     </row>
     <row r="56">
@@ -17956,7 +17956,7 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>18300</v>
+        <v>25825</v>
       </c>
     </row>
     <row r="57">
@@ -17966,7 +17966,7 @@
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>19775</v>
+        <v>27900</v>
       </c>
     </row>
     <row r="58">
@@ -17976,13 +17976,13 @@
         </is>
       </c>
       <c r="B58" s="7" t="n">
-        <v>21350</v>
+        <v>30125</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>Defaults: $800/mo by yr 3 (user), +12%/yr to yr 15 (income → ~$500k), +8%/yr after. Cap on Dashboard applies.</t>
+          <t>Defaults: $900/mo yr 1 (user, 2026), +12%/yr to yr 15 (income → ~$500k), +8%/yr after. Cap on Dashboard applies.</t>
         </is>
       </c>
     </row>
@@ -18395,7 +18395,7 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="58" t="inlineStr">
         <is>
-          <t>Year-by-year monthly schedule on Settings (defaults: $500 yr1, $800 by yr3, +12%/yr to yr15 as income scales to ~$500k, +8%/yr after), capped on the Dashboard. Projection applies the exact schedule.</t>
+          <t>Year-by-year monthly schedule on Settings (defaults: $900/mo yr1 per user 2026 update, +12%/yr to yr15 as income scales to ~$500k, +8%/yr after), capped on the Dashboard. Projection applies the exact schedule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Matrix v7: washout-conditional D rebound slice (MOD/AGG/VAGG)
- breadth signal: share of 18 sector ETFs above own 10m SMA (completed
  months, >=12 names required, fail-closed to standard cell)
- washout (<25%) grows the D-cell rebound equity slice by up to 10pp
  from TLT (VAGG caps at its 5pp TLT weight); CONS untouched
- signal recorded in ledger signals JSON; logger fetches breadth
  tickers with per-name failure tolerance
- workbook refreshed to v7 stats; 65 tests pass

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1598,7 +1598,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Matrix v6 (conditional-duration S, D-cell gold, R momentum tilt, regime-gated short book: oil in Deflation + energy equities in Stagflation behind a global include-shorts switch), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
+          <t>Matrix v7 (conditional-duration S, D-cell gold + washout-conditional rebound slice, R momentum tilt, regime-gated short book: oil in Deflation + energy equities in Stagflation behind a global include-shorts switch), monthly-only execution — intra-month mechanisms tested and rejected under honest T+1 modeling. Leveraged instruments simulated pre-2010. Out-of-sample framework validation: 1987-2007 replication. Forward: paper/ledger.csv.</t>
         </is>
       </c>
     </row>
@@ -1720,31 +1720,31 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>0.1528</v>
+        <v>0.1559</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>1.7335</v>
+        <v>1.7527</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>1.2456</v>
+        <v>1.2658</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>-0.1431</v>
+        <v>-0.143</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.2789</v>
+        <v>0.3274</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>0.2075</v>
+        <v>0.1545</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>0.36</v>
+        <v>0.3509</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>0.0002</v>
+        <v>0.0129</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>0.2861</v>
+        <v>0.2984</v>
       </c>
       <c r="K7" s="20" t="n">
         <v>0.1833</v>
@@ -1757,31 +1757,31 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>0.2408</v>
+        <v>0.2461</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>1.2244</v>
+        <v>1.2515</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>0.9427</v>
+        <v>0.9688</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0.3375</v>
+        <v>-0.3338</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>0.5864</v>
+        <v>0.6321</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>0.38</v>
+        <v>0.3177</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.9095</v>
+        <v>0.9175</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0.2531</v>
+        <v>-0.2463</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.4978</v>
+        <v>0.5163</v>
       </c>
       <c r="K8" s="18" t="n">
         <v>0.217</v>
@@ -1794,31 +1794,31 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>0.338</v>
+        <v>0.3436</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.1173</v>
+        <v>1.1346</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>0.8657</v>
+        <v>0.8812</v>
       </c>
       <c r="E9" s="20" t="n">
         <v>-0.489</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.9979</v>
+        <v>1.0393</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>0.4634</v>
+        <v>0.4131</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1.1018</v>
+        <v>1.1186</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>-0.3122</v>
+        <v>-0.3062</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>0.6196</v>
+        <v>0.6364</v>
       </c>
       <c r="K9" s="20" t="n">
         <v>0.4992</v>
@@ -18022,7 +18022,7 @@
     <row r="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Model Data — per-regime return statistics (matrix v6, monthly-only execution, Jun 2007–Aug 2026)</t>
+          <t>Model Data — per-regime return statistics (matrix v7, monthly-only execution, Jun 2007–Aug 2026)</t>
         </is>
       </c>
     </row>
@@ -18101,7 +18101,7 @@
         <v>0.00648</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>0.01783</v>
+        <v>0.01949</v>
       </c>
     </row>
     <row r="8">
@@ -18120,7 +18120,7 @@
         <v>0.00804</v>
       </c>
       <c r="E8" s="55" t="n">
-        <v>0.02193</v>
+        <v>0.02443</v>
       </c>
     </row>
     <row r="9">
@@ -18139,7 +18139,7 @@
         <v>0.00869</v>
       </c>
       <c r="E9" s="55" t="n">
-        <v>0.02982</v>
+        <v>0.03238</v>
       </c>
     </row>
     <row r="11">
@@ -18210,7 +18210,7 @@
         <v>0.02411</v>
       </c>
       <c r="E14" s="55" t="n">
-        <v>0.04132</v>
+        <v>0.03854</v>
       </c>
     </row>
     <row r="15">
@@ -18229,7 +18229,7 @@
         <v>0.03079</v>
       </c>
       <c r="E15" s="55" t="n">
-        <v>0.06388000000000001</v>
+        <v>0.05878</v>
       </c>
     </row>
     <row r="16">
@@ -18248,7 +18248,7 @@
         <v>0.03353</v>
       </c>
       <c r="E16" s="55" t="n">
-        <v>0.08375</v>
+        <v>0.08123</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Leveraged-ETF decay validated sim-vs-real; VAGG restated with ERX at 2x
Daily-reset sims track real products at 0.97-0.999 correlation with a
conservative bias (QLD -0.5, TQQQ -1.3, TMF -0.7%/yr vs real). ERX was
cut 3x->2x in Mar 2020; engine modeled 3x throughout — now 2x to match
the tradable product. VAGG restates 34.4->32.9% CAGR with a shallower
maxDD; other tiers unchanged; forward ledger never affected (marks to
real prices). Workbook refreshed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1794,34 +1794,34 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>0.3436</v>
+        <v>0.3285</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.1346</v>
+        <v>1.1241</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>0.8812</v>
+        <v>0.8825</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>-0.489</v>
+        <v>-0.4693</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>1.0393</v>
+        <v>0.9814000000000001</v>
       </c>
       <c r="G9" s="20" t="n">
         <v>0.4131</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1.1186</v>
+        <v>1.2807</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>-0.3062</v>
+        <v>-0.3418</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>0.6364</v>
+        <v>0.5962</v>
       </c>
       <c r="K9" s="20" t="n">
-        <v>0.4992</v>
+        <v>0.3673</v>
       </c>
     </row>
     <row r="10">
@@ -18133,7 +18133,7 @@
         <v>0.05004</v>
       </c>
       <c r="C9" s="55" t="n">
-        <v>0.01867</v>
+        <v>0.01582</v>
       </c>
       <c r="D9" s="55" t="n">
         <v>0.00869</v>
@@ -18242,7 +18242,7 @@
         <v>0.13741</v>
       </c>
       <c r="C16" s="55" t="n">
-        <v>0.07905</v>
+        <v>0.06832000000000001</v>
       </c>
       <c r="D16" s="55" t="n">
         <v>0.03353</v>

</xml_diff>

<commit_message>
Leverage audit: all products verified by realized beta; SCO restated to hybrid
QLD/TQQQ/TMF unchanged at stated leverage their whole lives; ERX/ERY
2x since Mar 2020 as restated. SCO's realized beta vs USO drifted to
-1.3 (basis, not leverage: USO restructured 2020); Apr 2020 divergence
(synthetic +72% vs real -7%) makes the synthetic model dishonest, so
the stats engine now uses real SCO from inception. VAGG 32.9->32.4,
MOD 15.6->15.3, AGG 24.6->24.2; workbook refreshed; 65 tests pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1720,31 +1720,31 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>0.1559</v>
+        <v>0.1534</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>1.7527</v>
+        <v>1.7215</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>1.2658</v>
+        <v>1.2463</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>-0.143</v>
+        <v>-0.1433</v>
       </c>
       <c r="F7" s="21" t="n">
-        <v>0.3274</v>
+        <v>0.3271</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>0.1545</v>
+        <v>0.1463</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>0.3509</v>
+        <v>0.2998</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>0.0129</v>
+        <v>0.0115</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>0.2984</v>
+        <v>0.3012</v>
       </c>
       <c r="K7" s="20" t="n">
         <v>0.1833</v>
@@ -1757,31 +1757,31 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>0.2461</v>
+        <v>0.242</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>1.2515</v>
+        <v>1.2306</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>0.9688</v>
+        <v>0.9532</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>-0.3338</v>
+        <v>-0.3342</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>0.6321</v>
+        <v>0.6317</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>0.3177</v>
+        <v>0.3038</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.9175</v>
+        <v>0.8095</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>-0.2463</v>
+        <v>-0.2478</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.5163</v>
+        <v>0.5212</v>
       </c>
       <c r="K8" s="18" t="n">
         <v>0.217</v>
@@ -1794,31 +1794,31 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>0.3285</v>
+        <v>0.3242</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>1.1241</v>
+        <v>1.1091</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>0.8825</v>
+        <v>0.8711</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>-0.4693</v>
+        <v>-0.4696</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>0.9814000000000001</v>
+        <v>0.981</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>0.4131</v>
+        <v>0.3983</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>1.2807</v>
+        <v>1.1519</v>
       </c>
       <c r="I9" s="20" t="n">
-        <v>-0.3418</v>
+        <v>-0.3432</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>0.5962</v>
+        <v>0.6012999999999999</v>
       </c>
       <c r="K9" s="20" t="n">
         <v>0.3673</v>
@@ -18101,7 +18101,7 @@
         <v>0.00648</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>0.01949</v>
+        <v>0.01795</v>
       </c>
     </row>
     <row r="8">
@@ -18120,7 +18120,7 @@
         <v>0.00804</v>
       </c>
       <c r="E8" s="55" t="n">
-        <v>0.02443</v>
+        <v>0.02203</v>
       </c>
     </row>
     <row r="9">
@@ -18139,7 +18139,7 @@
         <v>0.00869</v>
       </c>
       <c r="E9" s="55" t="n">
-        <v>0.03238</v>
+        <v>0.02989</v>
       </c>
     </row>
     <row r="11">
@@ -18210,7 +18210,7 @@
         <v>0.02411</v>
       </c>
       <c r="E14" s="55" t="n">
-        <v>0.03854</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="15">
@@ -18229,7 +18229,7 @@
         <v>0.03079</v>
       </c>
       <c r="E15" s="55" t="n">
-        <v>0.05878</v>
+        <v>0.05344</v>
       </c>
     </row>
     <row r="16">
@@ -18248,7 +18248,7 @@
         <v>0.03353</v>
       </c>
       <c r="E16" s="55" t="n">
-        <v>0.08123</v>
+        <v>0.07621</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Contribution schedule rebuilt to user's decade anchors
Yr1 $1,500/mo, +20%/yr through yr 5 (no-kids ramp), +7%/yr after:
crosses $5k/mo mid-30s, $7k early 40s, $12.9k at 50. Cap raised to
$25k. Dashboard default and runbook updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1144,7 +1144,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Age-based risk glide with regime-conditional return engine  |  Backtest Jun 2007–Aug 2026  |  Prepared August 21, 2026  |  Forward ledger live</t>
+          <t>Age-based risk glide with regime-conditional return engine  |  Backtest Jun 2007–Aug 2026  |  Prepared August 26, 2026  |  Forward ledger live</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>900</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="9">
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="10">
@@ -17596,7 +17596,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>1000</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="21">
@@ -17606,7 +17606,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>1125</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="22">
@@ -17616,7 +17616,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>1275</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="23">
@@ -17626,7 +17626,7 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>1425</v>
+        <v>3100</v>
       </c>
     </row>
     <row r="24">
@@ -17636,7 +17636,7 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>1575</v>
+        <v>3325</v>
       </c>
     </row>
     <row r="25">
@@ -17646,7 +17646,7 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>1775</v>
+        <v>3550</v>
       </c>
     </row>
     <row r="26">
@@ -17656,7 +17656,7 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>2000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="27">
@@ -17666,7 +17666,7 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>2225</v>
+        <v>4075</v>
       </c>
     </row>
     <row r="28">
@@ -17676,7 +17676,7 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>2500</v>
+        <v>4350</v>
       </c>
     </row>
     <row r="29">
@@ -17686,7 +17686,7 @@
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>2800</v>
+        <v>4675</v>
       </c>
     </row>
     <row r="30">
@@ -17696,7 +17696,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>3125</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="31">
@@ -17706,7 +17706,7 @@
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>3500</v>
+        <v>5350</v>
       </c>
     </row>
     <row r="32">
@@ -17716,7 +17716,7 @@
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>3925</v>
+        <v>5725</v>
       </c>
     </row>
     <row r="33">
@@ -17726,7 +17726,7 @@
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>4400</v>
+        <v>6125</v>
       </c>
     </row>
     <row r="34">
@@ -17736,7 +17736,7 @@
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>4750</v>
+        <v>6550</v>
       </c>
     </row>
     <row r="35">
@@ -17746,7 +17746,7 @@
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>5125</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="36">
@@ -17756,7 +17756,7 @@
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>5550</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="37">
@@ -17766,7 +17766,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>5975</v>
+        <v>8025</v>
       </c>
     </row>
     <row r="38">
@@ -17776,7 +17776,7 @@
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>6475</v>
+        <v>8575</v>
       </c>
     </row>
     <row r="39">
@@ -17786,7 +17786,7 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>6975</v>
+        <v>9175</v>
       </c>
     </row>
     <row r="40">
@@ -17796,7 +17796,7 @@
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>7550</v>
+        <v>9825</v>
       </c>
     </row>
     <row r="41">
@@ -17806,7 +17806,7 @@
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>8150</v>
+        <v>10525</v>
       </c>
     </row>
     <row r="42">
@@ -17816,7 +17816,7 @@
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>8800</v>
+        <v>11250</v>
       </c>
     </row>
     <row r="43">
@@ -17826,7 +17826,7 @@
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>9500</v>
+        <v>12025</v>
       </c>
     </row>
     <row r="44">
@@ -17836,7 +17836,7 @@
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>10250</v>
+        <v>12875</v>
       </c>
     </row>
     <row r="45">
@@ -17846,7 +17846,7 @@
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>11075</v>
+        <v>13775</v>
       </c>
     </row>
     <row r="46">
@@ -17856,7 +17856,7 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>11950</v>
+        <v>14750</v>
       </c>
     </row>
     <row r="47">
@@ -17866,7 +17866,7 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>12925</v>
+        <v>15775</v>
       </c>
     </row>
     <row r="48">
@@ -17876,7 +17876,7 @@
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>13950</v>
+        <v>16875</v>
       </c>
     </row>
     <row r="49">
@@ -17886,7 +17886,7 @@
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>15075</v>
+        <v>18075</v>
       </c>
     </row>
     <row r="50">
@@ -17896,7 +17896,7 @@
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>16275</v>
+        <v>19325</v>
       </c>
     </row>
     <row r="51">
@@ -17906,7 +17906,7 @@
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>17575</v>
+        <v>20675</v>
       </c>
     </row>
     <row r="52">
@@ -17916,7 +17916,7 @@
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>18975</v>
+        <v>22125</v>
       </c>
     </row>
     <row r="53">
@@ -17926,7 +17926,7 @@
         </is>
       </c>
       <c r="B53" s="7" t="n">
-        <v>20500</v>
+        <v>23675</v>
       </c>
     </row>
     <row r="54">
@@ -17936,7 +17936,7 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>22150</v>
+        <v>25325</v>
       </c>
     </row>
     <row r="55">
@@ -17946,7 +17946,7 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>23900</v>
+        <v>27100</v>
       </c>
     </row>
     <row r="56">
@@ -17956,7 +17956,7 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>25825</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="57">
@@ -17966,7 +17966,7 @@
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>27900</v>
+        <v>31025</v>
       </c>
     </row>
     <row r="58">
@@ -17976,13 +17976,13 @@
         </is>
       </c>
       <c r="B58" s="7" t="n">
-        <v>30125</v>
+        <v>33200</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>Defaults: $900/mo yr 1 (user, 2026), +12%/yr to yr 15 (income → ~$500k), +8%/yr after. Cap on Dashboard applies.</t>
+          <t>Defaults: $1,500/mo yr 1 (user, 2026); +20%/yr thru yr 5 (no-kids ramp), +7%/yr after — crosses $5k/mo early-mid 30s, $7k entering 40s, $10k+ mid-40s on. Cap on Dashboard applies.</t>
         </is>
       </c>
     </row>
@@ -18395,7 +18395,7 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="58" t="inlineStr">
         <is>
-          <t>Year-by-year monthly schedule on Settings (defaults: $900/mo yr1 per user 2026 update, +12%/yr to yr15 as income scales to ~$500k, +8%/yr after), capped on the Dashboard. Projection applies the exact schedule.</t>
+          <t>Year-by-year monthly schedule on Settings (defaults: $1,500/mo yr1 per user 2026 update; +20%/yr through yr5, +7%/yr after — anchored to user decade targets: &gt;$5k/mo in 30s, &gt;$7k in 40s, &gt;$10k in 50s), capped on the Dashboard. Projection applies the exact schedule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: 13-stage editable contribution ramp + fully labeled charts
- ramp is now an assumption: 13 three-year stages, each with a yellow
  growth-rate input; year-by-year schedule is formula-driven off the
  stage table (yr1 links to Dashboard); defaults 35% ages 26-28 then
  tapering 15->5%, honoring user anchors
- all three charts get axis titles, number formats, visible axes, and
  data labels (bar charts) / decade tick spacing (wealth path)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -535,6 +535,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -545,7 +546,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Month</a:t>
+                  <a:t>Months from start (age 25 -&gt; 65)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -555,12 +556,15 @@
         <minorTickMark val="none"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="60"/>
+        <tickMarkSkip val="60"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -572,12 +576,13 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Balance ($)</a:t>
+                  <a:t>Account balance ($)</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -641,6 +646,10 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.0%"/>
+          <showVal val="1"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -650,7 +659,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Portfolio / benchmark</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -661,8 +686,25 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Compound annual return</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -718,6 +760,10 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <numFmt formatCode="$#,##0"/>
+          <showVal val="1"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -727,7 +773,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Strategy / benchmark</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -738,8 +800,25 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>After-tax balance at end age ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -17572,11 +17651,15 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Contribution schedule — monthly $ by year (edit freely; year 1 links to Dashboard)</t>
+          <t>Contribution schedule — driven by the RAMP STAGES table (edit the yellow rates)</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
       <c r="C18" s="4" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
@@ -17588,6 +17671,21 @@
         <f>Dashboard!$C$8</f>
         <v/>
       </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Ramp stage</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>From yr</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Growth %/yr</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
@@ -17595,8 +17693,20 @@
           <t>Year 2</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
-        <v>1800</v>
+      <c r="B20" s="52">
+        <f>ROUND(B19*(1+INDEX($F$20:$F$32,MATCH(2,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>Ages 26-28</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="21">
@@ -17605,8 +17715,20 @@
           <t>Year 3</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n">
-        <v>2150</v>
+      <c r="B21" s="52">
+        <f>ROUND(B20*(1+INDEX($F$20:$F$32,MATCH(3,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Ages 29-31</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="22">
@@ -17615,8 +17737,20 @@
           <t>Year 4</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
-        <v>2600</v>
+      <c r="B22" s="52">
+        <f>ROUND(B21*(1+INDEX($F$20:$F$32,MATCH(4,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Ages 32-34</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="23">
@@ -17625,8 +17759,20 @@
           <t>Year 5</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n">
-        <v>3100</v>
+      <c r="B23" s="52">
+        <f>ROUND(B22*(1+INDEX($F$20:$F$32,MATCH(5,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Ages 35-37</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="24">
@@ -17635,8 +17781,20 @@
           <t>Year 6</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n">
-        <v>3325</v>
+      <c r="B24" s="52">
+        <f>ROUND(B23*(1+INDEX($F$20:$F$32,MATCH(6,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Ages 38-40</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="n">
+        <v>14</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="25">
@@ -17645,8 +17803,20 @@
           <t>Year 7</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
-        <v>3550</v>
+      <c r="B25" s="52">
+        <f>ROUND(B24*(1+INDEX($F$20:$F$32,MATCH(7,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Ages 41-43</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="n">
+        <v>17</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -17655,8 +17825,20 @@
           <t>Year 8</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n">
-        <v>3800</v>
+      <c r="B26" s="52">
+        <f>ROUND(B25*(1+INDEX($F$20:$F$32,MATCH(8,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Ages 44-46</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -17665,8 +17847,20 @@
           <t>Year 9</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n">
-        <v>4075</v>
+      <c r="B27" s="52">
+        <f>ROUND(B26*(1+INDEX($F$20:$F$32,MATCH(9,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Ages 47-49</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="n">
+        <v>23</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -17675,8 +17869,20 @@
           <t>Year 10</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n">
-        <v>4350</v>
+      <c r="B28" s="52">
+        <f>ROUND(B27*(1+INDEX($F$20:$F$32,MATCH(10,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>Ages 50-52</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="n">
+        <v>26</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="29">
@@ -17685,8 +17891,20 @@
           <t>Year 11</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
-        <v>4675</v>
+      <c r="B29" s="52">
+        <f>ROUND(B28*(1+INDEX($F$20:$F$32,MATCH(11,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Ages 53-55</t>
+        </is>
+      </c>
+      <c r="E29" s="27" t="n">
+        <v>29</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="30">
@@ -17695,8 +17913,20 @@
           <t>Year 12</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
-        <v>5000</v>
+      <c r="B30" s="52">
+        <f>ROUND(B29*(1+INDEX($F$20:$F$32,MATCH(12,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Ages 56-58</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="31">
@@ -17705,8 +17935,20 @@
           <t>Year 13</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
-        <v>5350</v>
+      <c r="B31" s="52">
+        <f>ROUND(B30*(1+INDEX($F$20:$F$32,MATCH(13,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Ages 59-61</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="n">
+        <v>35</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="32">
@@ -17715,8 +17957,20 @@
           <t>Year 14</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n">
-        <v>5725</v>
+      <c r="B32" s="52">
+        <f>ROUND(B31*(1+INDEX($F$20:$F$32,MATCH(14,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Ages 62-64</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="n">
+        <v>38</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="33">
@@ -17725,8 +17979,9 @@
           <t>Year 15</t>
         </is>
       </c>
-      <c r="B33" s="7" t="n">
-        <v>6125</v>
+      <c r="B33" s="52">
+        <f>ROUND(B32*(1+INDEX($F$20:$F$32,MATCH(15,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -17735,8 +17990,9 @@
           <t>Year 16</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n">
-        <v>6550</v>
+      <c r="B34" s="52">
+        <f>ROUND(B33*(1+INDEX($F$20:$F$32,MATCH(16,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -17745,8 +18001,9 @@
           <t>Year 17</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n">
-        <v>7000</v>
+      <c r="B35" s="52">
+        <f>ROUND(B34*(1+INDEX($F$20:$F$32,MATCH(17,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -17755,8 +18012,9 @@
           <t>Year 18</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
-        <v>7500</v>
+      <c r="B36" s="52">
+        <f>ROUND(B35*(1+INDEX($F$20:$F$32,MATCH(18,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -17765,8 +18023,9 @@
           <t>Year 19</t>
         </is>
       </c>
-      <c r="B37" s="7" t="n">
-        <v>8025</v>
+      <c r="B37" s="52">
+        <f>ROUND(B36*(1+INDEX($F$20:$F$32,MATCH(19,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -17775,8 +18034,9 @@
           <t>Year 20</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n">
-        <v>8575</v>
+      <c r="B38" s="52">
+        <f>ROUND(B37*(1+INDEX($F$20:$F$32,MATCH(20,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -17785,8 +18045,9 @@
           <t>Year 21</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n">
-        <v>9175</v>
+      <c r="B39" s="52">
+        <f>ROUND(B38*(1+INDEX($F$20:$F$32,MATCH(21,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -17795,8 +18056,9 @@
           <t>Year 22</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n">
-        <v>9825</v>
+      <c r="B40" s="52">
+        <f>ROUND(B39*(1+INDEX($F$20:$F$32,MATCH(22,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -17805,8 +18067,9 @@
           <t>Year 23</t>
         </is>
       </c>
-      <c r="B41" s="7" t="n">
-        <v>10525</v>
+      <c r="B41" s="52">
+        <f>ROUND(B40*(1+INDEX($F$20:$F$32,MATCH(23,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -17815,8 +18078,9 @@
           <t>Year 24</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n">
-        <v>11250</v>
+      <c r="B42" s="52">
+        <f>ROUND(B41*(1+INDEX($F$20:$F$32,MATCH(24,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -17825,8 +18089,9 @@
           <t>Year 25</t>
         </is>
       </c>
-      <c r="B43" s="7" t="n">
-        <v>12025</v>
+      <c r="B43" s="52">
+        <f>ROUND(B42*(1+INDEX($F$20:$F$32,MATCH(25,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -17835,8 +18100,9 @@
           <t>Year 26</t>
         </is>
       </c>
-      <c r="B44" s="7" t="n">
-        <v>12875</v>
+      <c r="B44" s="52">
+        <f>ROUND(B43*(1+INDEX($F$20:$F$32,MATCH(26,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -17845,8 +18111,9 @@
           <t>Year 27</t>
         </is>
       </c>
-      <c r="B45" s="7" t="n">
-        <v>13775</v>
+      <c r="B45" s="52">
+        <f>ROUND(B44*(1+INDEX($F$20:$F$32,MATCH(27,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -17855,8 +18122,9 @@
           <t>Year 28</t>
         </is>
       </c>
-      <c r="B46" s="7" t="n">
-        <v>14750</v>
+      <c r="B46" s="52">
+        <f>ROUND(B45*(1+INDEX($F$20:$F$32,MATCH(28,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -17865,8 +18133,9 @@
           <t>Year 29</t>
         </is>
       </c>
-      <c r="B47" s="7" t="n">
-        <v>15775</v>
+      <c r="B47" s="52">
+        <f>ROUND(B46*(1+INDEX($F$20:$F$32,MATCH(29,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -17875,8 +18144,9 @@
           <t>Year 30</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n">
-        <v>16875</v>
+      <c r="B48" s="52">
+        <f>ROUND(B47*(1+INDEX($F$20:$F$32,MATCH(30,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -17885,8 +18155,9 @@
           <t>Year 31</t>
         </is>
       </c>
-      <c r="B49" s="7" t="n">
-        <v>18075</v>
+      <c r="B49" s="52">
+        <f>ROUND(B48*(1+INDEX($F$20:$F$32,MATCH(31,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -17895,8 +18166,9 @@
           <t>Year 32</t>
         </is>
       </c>
-      <c r="B50" s="7" t="n">
-        <v>19325</v>
+      <c r="B50" s="52">
+        <f>ROUND(B49*(1+INDEX($F$20:$F$32,MATCH(32,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -17905,8 +18177,9 @@
           <t>Year 33</t>
         </is>
       </c>
-      <c r="B51" s="7" t="n">
-        <v>20675</v>
+      <c r="B51" s="52">
+        <f>ROUND(B50*(1+INDEX($F$20:$F$32,MATCH(33,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -17915,8 +18188,9 @@
           <t>Year 34</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n">
-        <v>22125</v>
+      <c r="B52" s="52">
+        <f>ROUND(B51*(1+INDEX($F$20:$F$32,MATCH(34,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -17925,8 +18199,9 @@
           <t>Year 35</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n">
-        <v>23675</v>
+      <c r="B53" s="52">
+        <f>ROUND(B52*(1+INDEX($F$20:$F$32,MATCH(35,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -17935,8 +18210,9 @@
           <t>Year 36</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n">
-        <v>25325</v>
+      <c r="B54" s="52">
+        <f>ROUND(B53*(1+INDEX($F$20:$F$32,MATCH(36,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="55">
@@ -17945,8 +18221,9 @@
           <t>Year 37</t>
         </is>
       </c>
-      <c r="B55" s="7" t="n">
-        <v>27100</v>
+      <c r="B55" s="52">
+        <f>ROUND(B54*(1+INDEX($F$20:$F$32,MATCH(37,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -17955,8 +18232,9 @@
           <t>Year 38</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n">
-        <v>29000</v>
+      <c r="B56" s="52">
+        <f>ROUND(B55*(1+INDEX($F$20:$F$32,MATCH(38,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="57">
@@ -17965,8 +18243,9 @@
           <t>Year 39</t>
         </is>
       </c>
-      <c r="B57" s="7" t="n">
-        <v>31025</v>
+      <c r="B57" s="52">
+        <f>ROUND(B56*(1+INDEX($F$20:$F$32,MATCH(39,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -17975,14 +18254,15 @@
           <t>Year 40</t>
         </is>
       </c>
-      <c r="B58" s="7" t="n">
-        <v>33200</v>
+      <c r="B58" s="52">
+        <f>ROUND(B57*(1+INDEX($F$20:$F$32,MATCH(40,$E$20:$E$32,1)))/25,0)*25</f>
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>Defaults: $1,500/mo yr 1 (user, 2026); +20%/yr thru yr 5 (no-kids ramp), +7%/yr after — crosses $5k/mo early-mid 30s, $7k entering 40s, $10k+ mid-40s on. Cap on Dashboard applies.</t>
+          <t>Yr 1 links to the Dashboard; every later year = prior year x (1 + its stage rate). Change the 13 yellow stage rates to reshape the whole ramp. Defaults honor the user's anchors: 35%/yr ages 26-28 (no kids), then tapering 15%-&gt;5%; crosses $5k/mo ~age 31, $7k ~34, cap ($25k, Dashboard) binds early 50s.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Contribution cap raised to 40k; fifties run uncapped
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBnnwzPLx94vYYG3d4vP48
</commit_message>
<xml_diff>
--- a/GrowthProjection.xlsx
+++ b/GrowthProjection.xlsx
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>25000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="10">
@@ -18262,7 +18262,7 @@
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>Yr 1 links to the Dashboard; every later year = prior year x (1 + its stage rate). Change the 13 yellow stage rates to reshape the whole ramp. Defaults honor the user's anchors: 35%/yr ages 26-28 (no kids), then tapering 15%-&gt;5%; crosses $5k/mo ~age 31, $7k ~34, cap ($25k, Dashboard) binds early 50s.</t>
+          <t>Yr 1 links to the Dashboard; every later year = prior year x (1 + its stage rate). Change the 13 yellow stage rates to reshape the whole ramp. Defaults honor the user's anchors: 35%/yr ages 26-28 (no kids), then tapering 15%-&gt;5%; crosses $5k/mo ~age 31, $7k ~34; cap ($40k, Dashboard) leaves the entire 50s uncapped and binds only ~age 62+.</t>
         </is>
       </c>
     </row>

</xml_diff>